<commit_message>
letter work post first submission
</commit_message>
<xml_diff>
--- a/cases/Fault_Cases/SMIB_RL_Line_DrCui.xlsx
+++ b/cases/Fault_Cases/SMIB_RL_Line_DrCui.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aali27/Work/repos/emt_simulator_basic/cases/SMIB_Chow/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aali27/Work/repos/emt_simulator_basic/cases/Fault_Cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{667073E5-878B-594A-A906-1397B2CE7C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84718297-98EB-8344-ACB7-5102A469FC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="30240" windowHeight="17700" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -831,7 +831,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="H2">
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -1088,7 +1088,7 @@
         <v>110</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2">
         <v>0</v>

</xml_diff>